<commit_message>
Audit and publish college production cluster
</commit_message>
<xml_diff>
--- a/college-production-tracker.xlsx
+++ b/college-production-tracker.xlsx
@@ -1217,27 +1217,27 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Created + Audited</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Created + Audited</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Created + Audited</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Created + Audited</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Not Applicable</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update college production queue status
</commit_message>
<xml_diff>
--- a/college-production-tracker.xlsx
+++ b/college-production-tracker.xlsx
@@ -1308,7 +1308,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>IIM Nagpur</t>
+          <t>Amrita Vishwa Vidyapeetham</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -1340,7 +1340,7 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Amrita Vishwa Vidyapeetham</t>
+          <t>IIT Kanpur</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
@@ -1372,7 +1372,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>IIT Kanpur</t>
+          <t>JMI</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -1404,7 +1404,7 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>JMI</t>
+          <t>IIM Visakhapatnam</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
@@ -1436,7 +1436,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>IIM Visakhapatnam</t>
+          <t>IMT Ghaziabad</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -1468,7 +1468,7 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>IMT Ghaziabad</t>
+          <t>IIM Bodh Gaya</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
@@ -1500,7 +1500,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>IIM Bodh Gaya</t>
+          <t>CU</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
@@ -1532,7 +1532,7 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>CU</t>
+          <t>MICA</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
@@ -1564,7 +1564,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>MICA</t>
+          <t>IIM Sambalpur</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -1596,7 +1596,7 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>IIM Sambalpur</t>
+          <t>IIM Jammu</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
@@ -1628,7 +1628,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>IIM Jammu</t>
+          <t>UPES</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
@@ -1660,7 +1660,7 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>UPES</t>
+          <t>Great Lakes Chennai</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
@@ -1692,7 +1692,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Great Lakes Chennai</t>
+          <t>IIM Shillong</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
@@ -1724,7 +1724,7 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>IIM Shillong</t>
+          <t>TAPMI Manipal</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
@@ -1756,7 +1756,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>TAPMI Manipal</t>
+          <t>IMI Delhi</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
@@ -1788,7 +1788,7 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>IMI Delhi</t>
+          <t>Jaipuria Institute of Management</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
@@ -1820,7 +1820,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Jaipuria Institute of Management</t>
+          <t>IMI Kolkata</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
@@ -1852,7 +1852,7 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>IMI Kolkata</t>
+          <t>GIM</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
@@ -1884,7 +1884,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>GIM</t>
+          <t>LPU</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
@@ -1916,7 +1916,7 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>LPU</t>
+          <t>XIM University</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
@@ -1948,7 +1948,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>XIM University</t>
+          <t>ICFAI Business School Hyderabad</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
@@ -1980,7 +1980,7 @@
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>ICFAI Business School Hyderabad</t>
+          <t>Thapar University</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
@@ -2012,7 +2012,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>Thapar University</t>
+          <t>IIT (ISM) Dhanbad</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
@@ -2044,7 +2044,7 @@
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>IIT (ISM) Dhanbad</t>
+          <t>Amity University</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
@@ -2076,7 +2076,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>Amity University</t>
+          <t>Great Lakes Gurgaon</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
@@ -2108,7 +2108,7 @@
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>Great Lakes Gurgaon</t>
+          <t>IIM Sirmaur</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
@@ -2140,7 +2140,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>IIM Sirmaur</t>
+          <t>Graphic Era</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
@@ -2172,7 +2172,7 @@
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>Graphic Era</t>
+          <t>Nirma University</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
@@ -2204,7 +2204,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>Nirma University</t>
+          <t>IRMA</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
@@ -2236,7 +2236,7 @@
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>IRMA</t>
+          <t>LIBA</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
@@ -2268,7 +2268,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>LIBA</t>
+          <t>SRMIST</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
@@ -2300,7 +2300,7 @@
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>SRMIST</t>
+          <t>Christ University</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
@@ -2332,7 +2332,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>Christ University</t>
+          <t>NIT Trichy</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
@@ -2364,7 +2364,7 @@
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>NIT Trichy</t>
+          <t>FORE School of Management</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
@@ -2396,7 +2396,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>FORE School of Management</t>
+          <t>BHU</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
@@ -2428,7 +2428,7 @@
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>BHU</t>
+          <t>BIMTECH</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
@@ -2460,7 +2460,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>BIMTECH</t>
+          <t>MNIT Jaipur</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
@@ -2492,7 +2492,7 @@
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>MNIT Jaipur</t>
+          <t>SIMATS</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
@@ -2524,7 +2524,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>SIMATS</t>
+          <t>IIM Amritsar</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
@@ -2556,7 +2556,7 @@
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>IIM Amritsar</t>
+          <t>K J Somaiya Institute of Management</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
@@ -2588,7 +2588,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>K J Somaiya Institute of Management</t>
+          <t>SOA University</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
@@ -2620,7 +2620,7 @@
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>SOA University</t>
+          <t>Jaipuria Lucknow</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
@@ -2652,7 +2652,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>Jaipuria Lucknow</t>
+          <t>KIIT</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
@@ -2684,7 +2684,7 @@
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>KIIT</t>
+          <t>AMU</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
@@ -2716,7 +2716,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>AMU</t>
+          <t>KL University</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
@@ -2748,7 +2748,7 @@
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>KL University</t>
+          <t>Alliance University</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
@@ -2780,7 +2780,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>Alliance University</t>
+          <t>IMT Nagpur</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
@@ -2812,7 +2812,7 @@
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>IMT Nagpur</t>
+          <t>JAIN University</t>
         </is>
       </c>
       <c r="B73" s="2" t="inlineStr">
@@ -2844,7 +2844,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>JAIN University</t>
+          <t>Jaipuria Noida</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
@@ -2876,7 +2876,7 @@
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>Jaipuria Noida</t>
+          <t>Welingkar (WeSchool)</t>
         </is>
       </c>
       <c r="B75" s="2" t="inlineStr">
@@ -2908,7 +2908,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>Welingkar (WeSchool)</t>
+          <t>GGSIPU</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
@@ -2940,7 +2940,7 @@
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>GGSIPU</t>
+          <t>BMU</t>
         </is>
       </c>
       <c r="B77" s="2" t="inlineStr">
@@ -2972,7 +2972,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>BMU</t>
+          <t>Chitkara University</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
@@ -3004,7 +3004,7 @@
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>Chitkara University</t>
+          <t>BBAU</t>
         </is>
       </c>
       <c r="B79" s="2" t="inlineStr">
@@ -3036,7 +3036,7 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>BBAU</t>
+          <t>TSM</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
@@ -3068,7 +3068,7 @@
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>TSM</t>
+          <t>MUJ</t>
         </is>
       </c>
       <c r="B81" s="2" t="inlineStr">
@@ -3100,7 +3100,7 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>MUJ</t>
+          <t>CUSAT</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
@@ -3132,7 +3132,7 @@
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>CUSAT</t>
+          <t>MMMUT</t>
         </is>
       </c>
       <c r="B83" s="2" t="inlineStr">
@@ -3164,7 +3164,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>MMMUT</t>
+          <t>PSG Tech</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
@@ -3196,7 +3196,7 @@
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>PSG Tech</t>
+          <t>NIT Calicut</t>
         </is>
       </c>
       <c r="B85" s="2" t="inlineStr">
@@ -3228,7 +3228,7 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>NIT Calicut</t>
+          <t>NDIM</t>
         </is>
       </c>
       <c r="B86" s="2" t="inlineStr">
@@ -3260,7 +3260,7 @@
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>NDIM</t>
+          <t>Jamia Hamdard</t>
         </is>
       </c>
       <c r="B87" s="2" t="inlineStr">
@@ -3292,7 +3292,7 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>Jamia Hamdard</t>
+          <t>Anna University</t>
         </is>
       </c>
       <c r="B88" s="2" t="inlineStr">
@@ -3324,7 +3324,7 @@
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>Anna University</t>
+          <t>PDEU</t>
         </is>
       </c>
       <c r="B89" s="2" t="inlineStr">
@@ -3356,7 +3356,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>PDEU</t>
+          <t>JIMS</t>
         </is>
       </c>
       <c r="B90" s="2" t="inlineStr">
@@ -3388,7 +3388,7 @@
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>JIMS</t>
+          <t>RBS</t>
         </is>
       </c>
       <c r="B91" s="2" t="inlineStr">
@@ -3420,7 +3420,7 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>RBS</t>
+          <t>PU</t>
         </is>
       </c>
       <c r="B92" s="2" t="inlineStr">
@@ -3452,7 +3452,7 @@
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
         <is>
-          <t>PU</t>
+          <t>ABV-IIITM Gwalior</t>
         </is>
       </c>
       <c r="B93" s="2" t="inlineStr">
@@ -3484,7 +3484,7 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>ABV-IIITM Gwalior</t>
+          <t>IMI Bhubaneswar</t>
         </is>
       </c>
       <c r="B94" s="2" t="inlineStr">
@@ -3516,7 +3516,7 @@
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
         <is>
-          <t>IMI Bhubaneswar</t>
+          <t>MANAGE</t>
         </is>
       </c>
       <c r="B95" s="2" t="inlineStr">
@@ -3548,7 +3548,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>MANAGE</t>
+          <t>BIM Trichy</t>
         </is>
       </c>
       <c r="B96" s="2" t="inlineStr">
@@ -3580,7 +3580,7 @@
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>BIM Trichy</t>
+          <t>BIT Mesra</t>
         </is>
       </c>
       <c r="B97" s="2" t="inlineStr">
@@ -3612,7 +3612,7 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>BIT Mesra</t>
+          <t>IIT Jodhpur</t>
         </is>
       </c>
       <c r="B98" s="2" t="inlineStr">
@@ -3644,7 +3644,7 @@
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>IIT Jodhpur</t>
+          <t>IMT Nagpur</t>
         </is>
       </c>
       <c r="B99" s="2" t="inlineStr">
@@ -3676,7 +3676,7 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>IMT Nagpur</t>
+          <t>Lucknow University</t>
         </is>
       </c>
       <c r="B100" s="2" t="inlineStr">
@@ -3708,7 +3708,7 @@
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
         <is>
-          <t>Lucknow University</t>
+          <t>IIM Nagpur</t>
         </is>
       </c>
       <c r="B101" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Release failed college and resume production queue
</commit_message>
<xml_diff>
--- a/college-production-tracker.xlsx
+++ b/college-production-tracker.xlsx
@@ -1313,27 +1313,27 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Created — Audit Pending</t>
+          <t>Needs Review</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Created — Audit Pending</t>
+          <t>Needs Review</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Created — Audit Pending</t>
+          <t>Needs Review</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>Created — Audit Pending</t>
+          <t>Needs Review</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>Created — Audit Pending</t>
+          <t>Needs Review</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Publish fully audited college production cluster
</commit_message>
<xml_diff>
--- a/college-production-tracker.xlsx
+++ b/college-production-tracker.xlsx
@@ -1377,27 +1377,27 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Created + Audited</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Created + Audited</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Not Applicable</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Not Applicable</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Not Applicable</t>
         </is>
       </c>
     </row>

</xml_diff>